<commit_message>
@ Scale-up: tea_scale_up.py on 551 model, metric-tonne SAF axis; regen figures + SI S9-1..S9-4
- tea_scale_up.py: read Pyrolysis_551_Scale* (was Jones_572_2MC) so panel (a) matches
  tea_scale_up_price_models.py / tea_pareto_front.py; xlsx export for plot_scale_up_from_xlsx.py
- tea_scale_up_price_models.py: SAF short ton -> metric tonne (x0.907185); xlsx export; figsize
- Regenerated scale-up figures incl. composite_scale_up_mjsp.png and Result/ xlsx
- SI.tex + SI md: Table S9-1 rebuilt (MJSP 1.638 -> 0.664), S9-2/S9-3 SAF column remapped,
  S9-4 caption 0.457 -> 0.414 MMt/yr
- _Scale_Up_Sensitivity.md: new section 1.3 + 2026-10-02 log

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Thc2pqJeabadCuAQ5dgUJZ
</commit_message>
<xml_diff>
--- a/Result/scale_up_base_summary.xlsx
+++ b/Result/scale_up_base_summary.xlsx
@@ -482,34 +482,34 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>0.042</v>
+        <v>0.041</v>
       </c>
       <c r="B2" t="n">
-        <v>1.039803682325185</v>
+        <v>1.152341275280172</v>
       </c>
       <c r="C2" t="n">
-        <v>1.285684130085952</v>
+        <v>1.283567261837519</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5775980254583015</v>
+        <v>0.6635974954308768</v>
       </c>
       <c r="E2" t="n">
-        <v>0.04930607371515114</v>
+        <v>0.03589294567451016</v>
       </c>
       <c r="F2" t="n">
-        <v>0.09491419190166595</v>
+        <v>0.1096142409569599</v>
       </c>
       <c r="G2" t="n">
-        <v>0.01232651842878778</v>
+        <v>0.00897323641862754</v>
       </c>
       <c r="H2" t="n">
-        <v>0.07211013280840854</v>
+        <v>0.07275359331573505</v>
       </c>
       <c r="I2" t="n">
-        <v>0.1650186240685903</v>
+        <v>0.1716175451515549</v>
       </c>
       <c r="J2" t="n">
-        <v>-1.817372387567797</v>
+        <v>-1.859954141293386</v>
       </c>
     </row>
     <row r="3">
@@ -517,191 +517,191 @@
         <v>0.104</v>
       </c>
       <c r="B3" t="n">
-        <v>0.7551419571214402</v>
+        <v>0.9356127133338452</v>
       </c>
       <c r="C3" t="n">
-        <v>1.270455183616835</v>
+        <v>1.268529249104018</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5362366736244915</v>
+        <v>0.5898860482225851</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01971944160435969</v>
+        <v>0.01435717815568198</v>
       </c>
       <c r="F3" t="n">
-        <v>0.07394790601634885</v>
+        <v>0.09289938806617754</v>
       </c>
       <c r="G3" t="n">
-        <v>0.004929860401089923</v>
+        <v>0.003589294538920496</v>
       </c>
       <c r="H3" t="n">
-        <v>0.04683367381035427</v>
+        <v>0.05362828311092976</v>
       </c>
       <c r="I3" t="n">
-        <v>0.153839815144869</v>
+        <v>0.1595033228269263</v>
       </c>
       <c r="J3" t="n">
-        <v>-1.8172968803463</v>
+        <v>-1.859954129544947</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>0.209</v>
+        <v>0.207</v>
       </c>
       <c r="B4" t="n">
-        <v>0.6706651608222605</v>
+        <v>0.8567862998312676</v>
       </c>
       <c r="C4" t="n">
-        <v>1.262198536318846</v>
+        <v>1.263494967299713</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5161472848983366</v>
+        <v>0.4674003164070594</v>
       </c>
       <c r="E4" t="n">
-        <v>0.009832642727171206</v>
+        <v>0.00661556248350053</v>
       </c>
       <c r="F4" t="n">
-        <v>0.06637033840840564</v>
+        <v>0.08550966401545897</v>
       </c>
       <c r="G4" t="n">
-        <v>0.002458160681792802</v>
+        <v>0.001653890620875132</v>
       </c>
       <c r="H4" t="n">
-        <v>0.03810149056778842</v>
+        <v>0.04606261324947975</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1492893656924521</v>
+        <v>0.1473349105567431</v>
       </c>
       <c r="J4" t="n">
-        <v>-1.816269116014985</v>
+        <v>-1.859954130909255</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>0.313</v>
+        <v>0.311</v>
       </c>
       <c r="B5" t="n">
-        <v>0.6461547296804573</v>
+        <v>0.800877129484036</v>
       </c>
       <c r="C5" t="n">
-        <v>1.263160683151052</v>
+        <v>1.261808772885304</v>
       </c>
       <c r="D5" t="n">
-        <v>0.4853120331203442</v>
+        <v>0.4063587469974212</v>
       </c>
       <c r="E5" t="n">
-        <v>0.006569951646792475</v>
+        <v>0.004785724838099601</v>
       </c>
       <c r="F5" t="n">
-        <v>0.06710736324938027</v>
+        <v>0.0832809959571254</v>
       </c>
       <c r="G5" t="n">
-        <v>0.001642487911698119</v>
+        <v>0.0011964312095249</v>
       </c>
       <c r="H5" t="n">
-        <v>0.03683865744808638</v>
+        <v>0.0440333603976125</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1465277544493706</v>
+        <v>0.1417949274996661</v>
       </c>
       <c r="J5" t="n">
-        <v>-1.817128434108455</v>
+        <v>-1.859953186793974</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>0.417</v>
+        <v>0.414</v>
       </c>
       <c r="B6" t="n">
-        <v>0.623096330229989</v>
+        <v>0.7498203834931433</v>
       </c>
       <c r="C6" t="n">
-        <v>1.262352147750016</v>
+        <v>1.260964599983058</v>
       </c>
       <c r="D6" t="n">
-        <v>0.4440528044426417</v>
+        <v>0.3678695293415354</v>
       </c>
       <c r="E6" t="n">
-        <v>0.004927620713661342</v>
+        <v>0.003589294525330143</v>
       </c>
       <c r="F6" t="n">
-        <v>0.06441104218571611</v>
+        <v>0.07794399385888497</v>
       </c>
       <c r="G6" t="n">
-        <v>0.001231905178415335</v>
+        <v>0.0008973236313325358</v>
       </c>
       <c r="H6" t="n">
-        <v>0.03466933144968873</v>
+        <v>0.04076664419210756</v>
       </c>
       <c r="I6" t="n">
-        <v>0.1426099191011648</v>
+        <v>0.1378414019251921</v>
       </c>
       <c r="J6" t="n">
-        <v>-1.817140535293566</v>
+        <v>-1.859954121278504</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>0.835</v>
+        <v>0.828</v>
       </c>
       <c r="B7" t="n">
-        <v>0.5889570976748495</v>
+        <v>0.7194430419437652</v>
       </c>
       <c r="C7" t="n">
-        <v>1.261163596153219</v>
+        <v>1.259688695038467</v>
       </c>
       <c r="D7" t="n">
-        <v>0.3664282391097197</v>
+        <v>0.326762348630424</v>
       </c>
       <c r="E7" t="n">
-        <v>0.002464008440853816</v>
+        <v>0.002603997338417961</v>
       </c>
       <c r="F7" t="n">
-        <v>0.06256821433739511</v>
+        <v>0.07741613708810154</v>
       </c>
       <c r="G7" t="n">
-        <v>0.000616002110213454</v>
+        <v>0.0006509993346044901</v>
       </c>
       <c r="H7" t="n">
-        <v>0.03251611138912446</v>
+        <v>0.04001006721325975</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1357413450036221</v>
+        <v>0.1342518979143957</v>
       </c>
       <c r="J7" t="n">
-        <v>-1.81717231962042</v>
+        <v>-1.859953186518556</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>1.252</v>
+        <v>1.243</v>
       </c>
       <c r="B8" t="n">
-        <v>0.5427428394297148</v>
+        <v>0.699726563169246</v>
       </c>
       <c r="C8" t="n">
-        <v>1.260779365003722</v>
+        <v>1.259253987944202</v>
       </c>
       <c r="D8" t="n">
-        <v>0.3281541428079763</v>
+        <v>0.3108015058515607</v>
       </c>
       <c r="E8" t="n">
-        <v>0.001642734809589841</v>
+        <v>0.001735998659336975</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0610158643561941</v>
+        <v>0.07858912849701169</v>
       </c>
       <c r="G8" t="n">
-        <v>0.0004106837023974603</v>
+        <v>0.0004339996648342437</v>
       </c>
       <c r="H8" t="n">
-        <v>0.03132929958289197</v>
+        <v>0.04016256357817433</v>
       </c>
       <c r="I8" t="n">
-        <v>0.1323486900076158</v>
+        <v>0.1329610756962726</v>
       </c>
       <c r="J8" t="n">
-        <v>-1.817187075278823</v>
+        <v>-1.85995411988849</v>
       </c>
     </row>
   </sheetData>

</xml_diff>